<commit_message>
Add 'FLOPs to Power' sheet inside the build-out workbook
The FLOPs conversion previously only lived in the separate scenarios workbook +
dashboard; the analyst works in Token_and_Data_Build_Out_v4_2.xlsx, so it looked
missing. Now write a "FLOPs to Power" snapshot sheet directly into that workbook
(next to Efficiency Overlay / Macro Levers): year, tokens/day, avg N, FLOPs/token,
FLOPs/day, fleet TFLOP/W, power GW.

research/refresh_flops_sheet_in_buildout.py does the surgical zip insert/overwrite
(idempotent), preserves every existing sheet's formula cache byte-for-byte, and
asserts the committed-base golden hash fdd0de9ef53c8247 before swapping the file in.
Static snapshot computed from the current Macro Levers tab; re-run to refresh.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Token_and_Data_Build_Out_v4_2.xlsx
+++ b/Token_and_Data_Build_Out_v4_2.xlsx
@@ -19,6 +19,7 @@
     <sheet name="Robo Bull" sheetId="4" r:id="rId4"/>
     <sheet name="Bear" sheetId="5" r:id="rId5"/>
     <sheet name="Macro Levers" sheetId="6" r:id="rId10"/>
+    <sheet name="FLOPs to Power" sheetId="7" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -17820,4 +17821,482 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="10"/>
+    <col min="2" max="7" width="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>FLOPs to Power (committed-base snapshot, FLOPs basis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Regenerate: python research/refresh_flops_sheet_in_buildout.py (reflects Macro Levers tab)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>tokens_per_day_T</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>avg_N_active_B</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FLOPs_per_token</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>FLOPs_per_day</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>fleet_TFLOP_per_W</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>power_GW</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>2025</v>
+      </c>
+      <c r="B4">
+        <v>134.9</v>
+      </c>
+      <c r="C4">
+        <v>297</v>
+      </c>
+      <c r="D4">
+        <v>5.944e+11</v>
+      </c>
+      <c r="E4">
+        <v>8.0197756e+25</v>
+      </c>
+      <c r="F4">
+        <v>9</v>
+      </c>
+      <c r="G4">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>2026</v>
+      </c>
+      <c r="B5">
+        <v>460.8</v>
+      </c>
+      <c r="C5">
+        <v>284</v>
+      </c>
+      <c r="D5">
+        <v>5.6857333e+11</v>
+      </c>
+      <c r="E5">
+        <v>2.6202362e+26</v>
+      </c>
+      <c r="F5">
+        <v>11</v>
+      </c>
+      <c r="G5">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>2027</v>
+      </c>
+      <c r="B6">
+        <v>763.6</v>
+      </c>
+      <c r="C6">
+        <v>271</v>
+      </c>
+      <c r="D6">
+        <v>5.4274667e+11</v>
+      </c>
+      <c r="E6">
+        <v>4.1444856e+26</v>
+      </c>
+      <c r="F6">
+        <v>14</v>
+      </c>
+      <c r="G6">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>2028</v>
+      </c>
+      <c r="B7">
+        <v>1359.8</v>
+      </c>
+      <c r="C7">
+        <v>258</v>
+      </c>
+      <c r="D7">
+        <v>5.1692e+11</v>
+      </c>
+      <c r="E7">
+        <v>7.0290923e+26</v>
+      </c>
+      <c r="F7">
+        <v>18</v>
+      </c>
+      <c r="G7">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>2029</v>
+      </c>
+      <c r="B8">
+        <v>2172.8</v>
+      </c>
+      <c r="C8">
+        <v>246</v>
+      </c>
+      <c r="D8">
+        <v>4.9109333e+11</v>
+      </c>
+      <c r="E8">
+        <v>1.0670445e+27</v>
+      </c>
+      <c r="F8">
+        <v>21.5</v>
+      </c>
+      <c r="G8">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>2030</v>
+      </c>
+      <c r="B9">
+        <v>3253.6</v>
+      </c>
+      <c r="C9">
+        <v>233</v>
+      </c>
+      <c r="D9">
+        <v>4.6526667e+11</v>
+      </c>
+      <c r="E9">
+        <v>1.5137842e+27</v>
+      </c>
+      <c r="F9">
+        <v>25</v>
+      </c>
+      <c r="G9">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>2031</v>
+      </c>
+      <c r="B10">
+        <v>4573</v>
+      </c>
+      <c r="C10">
+        <v>220</v>
+      </c>
+      <c r="D10">
+        <v>4.3944e+11</v>
+      </c>
+      <c r="E10">
+        <v>2.0095756e+27</v>
+      </c>
+      <c r="F10">
+        <v>28</v>
+      </c>
+      <c r="G10">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>2032</v>
+      </c>
+      <c r="B11">
+        <v>5901.4</v>
+      </c>
+      <c r="C11">
+        <v>207</v>
+      </c>
+      <c r="D11">
+        <v>4.1361333e+11</v>
+      </c>
+      <c r="E11">
+        <v>2.440905e+27</v>
+      </c>
+      <c r="F11">
+        <v>31</v>
+      </c>
+      <c r="G11">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>2033</v>
+      </c>
+      <c r="B12">
+        <v>7334.6</v>
+      </c>
+      <c r="C12">
+        <v>194</v>
+      </c>
+      <c r="D12">
+        <v>3.8778667e+11</v>
+      </c>
+      <c r="E12">
+        <v>2.8442663e+27</v>
+      </c>
+      <c r="F12">
+        <v>34</v>
+      </c>
+      <c r="G12">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>2034</v>
+      </c>
+      <c r="B13">
+        <v>8998.7</v>
+      </c>
+      <c r="C13">
+        <v>181</v>
+      </c>
+      <c r="D13">
+        <v>3.6196e+11</v>
+      </c>
+      <c r="E13">
+        <v>3.2571717e+27</v>
+      </c>
+      <c r="F13">
+        <v>37</v>
+      </c>
+      <c r="G13">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>2035</v>
+      </c>
+      <c r="B14">
+        <v>10620.4</v>
+      </c>
+      <c r="C14">
+        <v>168</v>
+      </c>
+      <c r="D14">
+        <v>3.3613333e+11</v>
+      </c>
+      <c r="E14">
+        <v>3.5698858e+27</v>
+      </c>
+      <c r="F14">
+        <v>40</v>
+      </c>
+      <c r="G14">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>2036</v>
+      </c>
+      <c r="B15">
+        <v>12433.3</v>
+      </c>
+      <c r="C15">
+        <v>155</v>
+      </c>
+      <c r="D15">
+        <v>3.1030667e+11</v>
+      </c>
+      <c r="E15">
+        <v>3.8581276e+27</v>
+      </c>
+      <c r="F15">
+        <v>42.9</v>
+      </c>
+      <c r="G15">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>2037</v>
+      </c>
+      <c r="B16">
+        <v>14482.7</v>
+      </c>
+      <c r="C16">
+        <v>142</v>
+      </c>
+      <c r="D16">
+        <v>2.8448e+11</v>
+      </c>
+      <c r="E16">
+        <v>4.120045e+27</v>
+      </c>
+      <c r="F16">
+        <v>45.7</v>
+      </c>
+      <c r="G16">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>2038</v>
+      </c>
+      <c r="B17">
+        <v>16709.1</v>
+      </c>
+      <c r="C17">
+        <v>129</v>
+      </c>
+      <c r="D17">
+        <v>2.5865333e+11</v>
+      </c>
+      <c r="E17">
+        <v>4.3218729e+27</v>
+      </c>
+      <c r="F17">
+        <v>48.6</v>
+      </c>
+      <c r="G17">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>2039</v>
+      </c>
+      <c r="B18">
+        <v>18373.4</v>
+      </c>
+      <c r="C18">
+        <v>116</v>
+      </c>
+      <c r="D18">
+        <v>2.3282667e+11</v>
+      </c>
+      <c r="E18">
+        <v>4.277828e+27</v>
+      </c>
+      <c r="F18">
+        <v>51.4</v>
+      </c>
+      <c r="G18">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>2040</v>
+      </c>
+      <c r="B19">
+        <v>20019.8</v>
+      </c>
+      <c r="C19">
+        <v>104</v>
+      </c>
+      <c r="D19">
+        <v>2.07e+11</v>
+      </c>
+      <c r="E19">
+        <v>4.1441009e+27</v>
+      </c>
+      <c r="F19">
+        <v>54.3</v>
+      </c>
+      <c r="G19">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>2041</v>
+      </c>
+      <c r="B20">
+        <v>21860.1</v>
+      </c>
+      <c r="C20">
+        <v>104</v>
+      </c>
+      <c r="D20">
+        <v>2.07e+11</v>
+      </c>
+      <c r="E20">
+        <v>4.5250457e+27</v>
+      </c>
+      <c r="F20">
+        <v>57.1</v>
+      </c>
+      <c r="G20">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>2042</v>
+      </c>
+      <c r="B21">
+        <v>23789.7</v>
+      </c>
+      <c r="C21">
+        <v>104</v>
+      </c>
+      <c r="D21">
+        <v>2.07e+11</v>
+      </c>
+      <c r="E21">
+        <v>4.9244656e+27</v>
+      </c>
+      <c r="F21">
+        <v>60</v>
+      </c>
+      <c r="G21">
+        <v>708</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add clean 'Duration Lens' presentation sheet to the workbook
A write-from-able summary tab in Token_and_Data_Build_Out_v4_2.xlsx: 7-step
narrative (the question -> tokens->FLOPs->power conversion with a live 2025/2035
worked example -> the tug-of-war -> token-base vs FLOPs-lens comparison -> a
chart-ready data block -> stress-test pointers -> the takeaway).

The conversion example and the chart block's FLOPs-demand line are LIVE-LINKED to
the 'FLOPs to Power' tab, so editing inputs there updates this sheet and any chart
built off A27:D45. Token base + supply are the locked committed snapshot.

Bold headers reuse an existing style (no styles.xml edit). Surgical zip insert;
golden hash fdd0de9ef53c8247 intact. Generator: research/build_duration_lens_sheet.py
(idempotent). Inserts as sheet 8 / rId12.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Token_and_Data_Build_Out_v4_2.xlsx
+++ b/Token_and_Data_Build_Out_v4_2.xlsx
@@ -20,6 +20,7 @@
     <sheet name="Bear" sheetId="5" r:id="rId5"/>
     <sheet name="Macro Levers" sheetId="6" r:id="rId10"/>
     <sheet name="FLOPs to Power" sheetId="7" r:id="rId11"/>
+    <sheet name="Duration Lens" sheetId="8" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -18545,4 +18546,579 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="52"/>
+    <col min="2" max="4" width="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="47" t="inlineStr">
+        <is>
+          <t>AI POWER DEMAND  —  THE DURATION LENS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Token base (committed headline) vs the FLOPs lens. A token's power cost varies ~50x by model, so convert tokens -&gt; FLOPs -&gt; power. Live mechanics + stress-test inputs are on the 'FLOPs to Power' tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="47" t="inlineStr">
+        <is>
+          <t>1. THE QUESTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>How big does AI power demand get, and how long does the shortage last? FLOPs/token = 2 x active params; that is the honest power unit a token-count model cannot see (routing/orchestration moves it).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="47" t="inlineStr">
+        <is>
+          <t>2. THE CONVERSION  (one row = one year; full live version on 'FLOPs to Power')</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="47" t="inlineStr">
+        <is>
+          <t>step</t>
+        </is>
+      </c>
+      <c r="B8" s="47" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C8" s="47" t="inlineStr">
+        <is>
+          <t>2035</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>tokens/day (T)</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>'FLOPs to Power'!B8</f>
+        <v>134.9222</v>
+      </c>
+      <c r="C9">
+        <f>'FLOPs to Power'!B18</f>
+        <v>10620.446</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>x  FLOPs/token (2 x N_active)</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>'FLOPs to Power'!F8</f>
+        <v>5.944e+11</v>
+      </c>
+      <c r="C10">
+        <f>'FLOPs to Power'!F18</f>
+        <v>3.3613333e+11</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>=  FLOPs/day</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>'FLOPs to Power'!G8</f>
+        <v>8.0197756e+25</v>
+      </c>
+      <c r="C11">
+        <f>'FLOPs to Power'!G18</f>
+        <v>3.5698858e+27</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>/  chip efficiency (TFLOP/W)</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>'FLOPs to Power'!E8</f>
+        <v>9</v>
+      </c>
+      <c r="C12">
+        <f>'FLOPs to Power'!E18</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>=  power (GW)</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>'FLOPs to Power'!I8</f>
+        <v>70</v>
+      </c>
+      <c r="C13">
+        <f>'FLOPs to Power'!I18</f>
+        <v>701.08822</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="47" t="inlineStr">
+        <is>
+          <t>3. THE TUG-OF-WAR  (why power grows ~10x, not ~176x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Tokens grow ~176x to 2042. But model size N falls ~3x (routing to smaller models) and chip TFLOP/W rises ~7x. Together they absorb most of it, so power grows ~10x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="47" t="inlineStr">
+        <is>
+          <t>4. TOKEN BASE  vs  FLOPs LENS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="47" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B19" s="47" t="inlineStr">
+        <is>
+          <t>Token base</t>
+        </is>
+      </c>
+      <c r="C19" s="47" t="inlineStr">
+        <is>
+          <t>FLOPs lens</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Peak gap (GW)</t>
+        </is>
+      </c>
+      <c r="B20">
+        <v>332</v>
+      </c>
+      <c r="C20">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Peak year</t>
+        </is>
+      </c>
+      <c r="B21">
+        <v>2029</v>
+      </c>
+      <c r="C21">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Demand floor 2042 (GW)</t>
+        </is>
+      </c>
+      <c r="B22">
+        <v>549</v>
+      </c>
+      <c r="C22">
+        <f>'FLOPs to Power'!I25</f>
+        <v>708</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Gap closes (overshoot)</t>
+        </is>
+      </c>
+      <c r="B23">
+        <v>2034</v>
+      </c>
+      <c r="C23">
+        <v>2036</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>timing / peak</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>duration / higher floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="47" t="inlineStr">
+        <is>
+          <t>5. CHART THIS  (select A27:D45, then Insert &gt; Line Chart)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="47" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B27" s="47" t="inlineStr">
+        <is>
+          <t>Token demand (GW)</t>
+        </is>
+      </c>
+      <c r="C27" s="47" t="inlineStr">
+        <is>
+          <t>FLOPs demand (GW)</t>
+        </is>
+      </c>
+      <c r="D27" s="47" t="inlineStr">
+        <is>
+          <t>Supply (GW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>2025</v>
+      </c>
+      <c r="B28">
+        <v>70</v>
+      </c>
+      <c r="C28">
+        <f>'FLOPs to Power'!I8</f>
+        <v>70</v>
+      </c>
+      <c r="D28">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>2026</v>
+      </c>
+      <c r="B29">
+        <v>219.2</v>
+      </c>
+      <c r="C29">
+        <f>'FLOPs to Power'!I9</f>
+        <v>187.1</v>
+      </c>
+      <c r="D29">
+        <v>85.4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>2027</v>
+      </c>
+      <c r="B30">
+        <v>305.7</v>
+      </c>
+      <c r="C30">
+        <f>'FLOPs to Power'!I10</f>
+        <v>232.6</v>
+      </c>
+      <c r="D30">
+        <v>104.2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>2028</v>
+      </c>
+      <c r="B31">
+        <v>427</v>
+      </c>
+      <c r="C31">
+        <f>'FLOPs to Power'!I11</f>
+        <v>306.8</v>
+      </c>
+      <c r="D31">
+        <v>135.4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>2029</v>
+      </c>
+      <c r="B32">
+        <v>508.5</v>
+      </c>
+      <c r="C32">
+        <f>'FLOPs to Power'!I12</f>
+        <v>389.9</v>
+      </c>
+      <c r="D32">
+        <v>176.1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>2030</v>
+      </c>
+      <c r="B33">
+        <v>548.9</v>
+      </c>
+      <c r="C33">
+        <f>'FLOPs to Power'!I13</f>
+        <v>475.7</v>
+      </c>
+      <c r="D33">
+        <v>228.9</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>2031</v>
+      </c>
+      <c r="B34">
+        <v>548.9</v>
+      </c>
+      <c r="C34">
+        <f>'FLOPs to Power'!I14</f>
+        <v>563.8</v>
+      </c>
+      <c r="D34">
+        <v>286.1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>2032</v>
+      </c>
+      <c r="B35">
+        <v>548.9</v>
+      </c>
+      <c r="C35">
+        <f>'FLOPs to Power'!I15</f>
+        <v>618.5</v>
+      </c>
+      <c r="D35">
+        <v>357.7</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>2033</v>
+      </c>
+      <c r="B36">
+        <v>548.9</v>
+      </c>
+      <c r="C36">
+        <f>'FLOPs to Power'!I16</f>
+        <v>657.2</v>
+      </c>
+      <c r="D36">
+        <v>447.1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>2034</v>
+      </c>
+      <c r="B37">
+        <v>548.9</v>
+      </c>
+      <c r="C37">
+        <f>'FLOPs to Power'!I17</f>
+        <v>691.5</v>
+      </c>
+      <c r="D37">
+        <v>558.8</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <v>2035</v>
+      </c>
+      <c r="B38">
+        <v>548.9</v>
+      </c>
+      <c r="C38">
+        <f>'FLOPs to Power'!I18</f>
+        <v>701.1</v>
+      </c>
+      <c r="D38">
+        <v>698.6</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <v>2036</v>
+      </c>
+      <c r="B39">
+        <v>548.9</v>
+      </c>
+      <c r="C39">
+        <f>'FLOPs to Power'!I19</f>
+        <v>707.2</v>
+      </c>
+      <c r="D39">
+        <v>803.3</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>2037</v>
+      </c>
+      <c r="B40">
+        <v>548.9</v>
+      </c>
+      <c r="C40">
+        <f>'FLOPs to Power'!I20</f>
+        <v>708</v>
+      </c>
+      <c r="D40">
+        <v>923.8</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <v>2038</v>
+      </c>
+      <c r="B41">
+        <v>548.9</v>
+      </c>
+      <c r="C41">
+        <f>'FLOPs to Power'!I21</f>
+        <v>708</v>
+      </c>
+      <c r="D41">
+        <v>1062.4</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>2039</v>
+      </c>
+      <c r="B42">
+        <v>548.9</v>
+      </c>
+      <c r="C42">
+        <f>'FLOPs to Power'!I22</f>
+        <v>708</v>
+      </c>
+      <c r="D42">
+        <v>1221.8</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>2040</v>
+      </c>
+      <c r="B43">
+        <v>548.9</v>
+      </c>
+      <c r="C43">
+        <f>'FLOPs to Power'!I23</f>
+        <v>708</v>
+      </c>
+      <c r="D43">
+        <v>1405</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <v>2041</v>
+      </c>
+      <c r="B44">
+        <v>548.9</v>
+      </c>
+      <c r="C44">
+        <f>'FLOPs to Power'!I24</f>
+        <v>708</v>
+      </c>
+      <c r="D44">
+        <v>1615.8</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <v>2042</v>
+      </c>
+      <c r="B45">
+        <v>548.9</v>
+      </c>
+      <c r="C45">
+        <f>'FLOPs to Power'!I25</f>
+        <v>708</v>
+      </c>
+      <c r="D45">
+        <v>1858.2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="47" t="inlineStr">
+        <is>
+          <t>6. STRESS-TEST IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Edit inputs on 'FLOPs to Power' (anchor, training share, N, TFLOP/W, retirement) — the FLOPs column above and this chart's FLOPs line update live. Broader levers on 'Macro Levers'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="47" t="inlineStr">
+        <is>
+          <t>7. THE TAKEAWAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>The FLOPs lens does NOT raise the peak (~278 vs 332). It raises the FLOOR (~708 vs 549, +29%) and extends the TIGHTNESS (gap closes ~2036 vs 2034). The power/grid/cooling case is about DURATION, not magnitude.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Tie-out fix: all 120 workbook formulas recompute to cached value
Audited every formula on the FLOPs to Power / Duration Lens / Macro Levers tabs by
independently re-evaluating against referenced cells. Fixed two drift sources on
Duration Lens so cache == formula exactly (recalc-on-open is now a no-op):
- live-linked chart/comparison cells wrapped in ROUND() so display and recompute
  agree (was: rounded cache vs full-precision formula)
- cache written at full native-float precision (was %.8g, drifted vs the %.10g
  cells it links to); coerce numpy->float so repr() emits valid XML
- step labels no longer start with '=' (unambiguously text, not formulas)

Result: 120/120 formulas tie out, 0 mismatches. Golden hash fdd0de9ef53c8247 intact.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Token_and_Data_Build_Out_v4_2.xlsx
+++ b/Token_and_Data_Build_Out_v4_2.xlsx
@@ -18621,67 +18621,67 @@
       </c>
       <c r="C9">
         <f>'FLOPs to Power'!B18</f>
-        <v>10620.446</v>
+        <v>10620.445661620677</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>x  FLOPs/token (2 x N_active)</t>
+          <t>x  FLOPs per token (2 x N_active)</t>
         </is>
       </c>
       <c r="B10">
         <f>'FLOPs to Power'!F8</f>
-        <v>5.944e+11</v>
+        <v>594400000000.0</v>
       </c>
       <c r="C10">
         <f>'FLOPs to Power'!F18</f>
-        <v>3.3613333e+11</v>
+        <v>336133333333.3334</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>=  FLOPs/day</t>
+          <t>-&gt;  FLOPs per day</t>
         </is>
       </c>
       <c r="B11">
         <f>'FLOPs to Power'!G8</f>
-        <v>8.0197756e+25</v>
+        <v>8.019775568e+25</v>
       </c>
       <c r="C11">
         <f>'FLOPs to Power'!G18</f>
-        <v>3.5698858e+27</v>
+        <v>3.569885801726098e+27</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>/  chip efficiency (TFLOP/W)</t>
+          <t>/  chip efficiency (TFLOP per W)</t>
         </is>
       </c>
       <c r="B12">
         <f>'FLOPs to Power'!E8</f>
-        <v>9</v>
+        <v>9.0</v>
       </c>
       <c r="C12">
         <f>'FLOPs to Power'!E18</f>
-        <v>40</v>
+        <v>40.0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>=  power (GW)</t>
+          <t>-&gt;  power (GW)</t>
         </is>
       </c>
       <c r="B13">
         <f>'FLOPs to Power'!I8</f>
-        <v>70</v>
+        <v>70.0</v>
       </c>
       <c r="C13">
         <f>'FLOPs to Power'!I18</f>
-        <v>701.08822</v>
+        <v>701.0882150060941</v>
       </c>
     </row>
     <row r="15">
@@ -18758,7 +18758,7 @@
         <v>549</v>
       </c>
       <c r="C22">
-        <f>'FLOPs to Power'!I25</f>
+        <f>ROUND('FLOPs to Power'!I25,0)</f>
         <v>708</v>
       </c>
     </row>
@@ -18826,14 +18826,14 @@
         <v>2025</v>
       </c>
       <c r="B28">
-        <v>70</v>
+        <v>70.0</v>
       </c>
       <c r="C28">
-        <f>'FLOPs to Power'!I8</f>
-        <v>70</v>
+        <f>ROUND('FLOPs to Power'!I8,1)</f>
+        <v>70.0</v>
       </c>
       <c r="D28">
-        <v>70</v>
+        <v>70.0</v>
       </c>
     </row>
     <row r="29">
@@ -18844,7 +18844,7 @@
         <v>219.2</v>
       </c>
       <c r="C29">
-        <f>'FLOPs to Power'!I9</f>
+        <f>ROUND('FLOPs to Power'!I9,1)</f>
         <v>187.1</v>
       </c>
       <c r="D29">
@@ -18859,7 +18859,7 @@
         <v>305.7</v>
       </c>
       <c r="C30">
-        <f>'FLOPs to Power'!I10</f>
+        <f>ROUND('FLOPs to Power'!I10,1)</f>
         <v>232.6</v>
       </c>
       <c r="D30">
@@ -18871,10 +18871,10 @@
         <v>2028</v>
       </c>
       <c r="B31">
-        <v>427</v>
+        <v>427.0</v>
       </c>
       <c r="C31">
-        <f>'FLOPs to Power'!I11</f>
+        <f>ROUND('FLOPs to Power'!I11,1)</f>
         <v>306.8</v>
       </c>
       <c r="D31">
@@ -18889,7 +18889,7 @@
         <v>508.5</v>
       </c>
       <c r="C32">
-        <f>'FLOPs to Power'!I12</f>
+        <f>ROUND('FLOPs to Power'!I12,1)</f>
         <v>389.9</v>
       </c>
       <c r="D32">
@@ -18904,7 +18904,7 @@
         <v>548.9</v>
       </c>
       <c r="C33">
-        <f>'FLOPs to Power'!I13</f>
+        <f>ROUND('FLOPs to Power'!I13,1)</f>
         <v>475.7</v>
       </c>
       <c r="D33">
@@ -18919,7 +18919,7 @@
         <v>548.9</v>
       </c>
       <c r="C34">
-        <f>'FLOPs to Power'!I14</f>
+        <f>ROUND('FLOPs to Power'!I14,1)</f>
         <v>563.8</v>
       </c>
       <c r="D34">
@@ -18934,7 +18934,7 @@
         <v>548.9</v>
       </c>
       <c r="C35">
-        <f>'FLOPs to Power'!I15</f>
+        <f>ROUND('FLOPs to Power'!I15,1)</f>
         <v>618.5</v>
       </c>
       <c r="D35">
@@ -18949,7 +18949,7 @@
         <v>548.9</v>
       </c>
       <c r="C36">
-        <f>'FLOPs to Power'!I16</f>
+        <f>ROUND('FLOPs to Power'!I16,1)</f>
         <v>657.2</v>
       </c>
       <c r="D36">
@@ -18964,7 +18964,7 @@
         <v>548.9</v>
       </c>
       <c r="C37">
-        <f>'FLOPs to Power'!I17</f>
+        <f>ROUND('FLOPs to Power'!I17,1)</f>
         <v>691.5</v>
       </c>
       <c r="D37">
@@ -18979,7 +18979,7 @@
         <v>548.9</v>
       </c>
       <c r="C38">
-        <f>'FLOPs to Power'!I18</f>
+        <f>ROUND('FLOPs to Power'!I18,1)</f>
         <v>701.1</v>
       </c>
       <c r="D38">
@@ -18994,7 +18994,7 @@
         <v>548.9</v>
       </c>
       <c r="C39">
-        <f>'FLOPs to Power'!I19</f>
+        <f>ROUND('FLOPs to Power'!I19,1)</f>
         <v>707.2</v>
       </c>
       <c r="D39">
@@ -19009,8 +19009,8 @@
         <v>548.9</v>
       </c>
       <c r="C40">
-        <f>'FLOPs to Power'!I20</f>
-        <v>708</v>
+        <f>ROUND('FLOPs to Power'!I20,1)</f>
+        <v>708.0</v>
       </c>
       <c r="D40">
         <v>923.8</v>
@@ -19024,8 +19024,8 @@
         <v>548.9</v>
       </c>
       <c r="C41">
-        <f>'FLOPs to Power'!I21</f>
-        <v>708</v>
+        <f>ROUND('FLOPs to Power'!I21,1)</f>
+        <v>708.0</v>
       </c>
       <c r="D41">
         <v>1062.4</v>
@@ -19039,8 +19039,8 @@
         <v>548.9</v>
       </c>
       <c r="C42">
-        <f>'FLOPs to Power'!I22</f>
-        <v>708</v>
+        <f>ROUND('FLOPs to Power'!I22,1)</f>
+        <v>708.0</v>
       </c>
       <c r="D42">
         <v>1221.8</v>
@@ -19054,11 +19054,11 @@
         <v>548.9</v>
       </c>
       <c r="C43">
-        <f>'FLOPs to Power'!I23</f>
-        <v>708</v>
+        <f>ROUND('FLOPs to Power'!I23,1)</f>
+        <v>708.0</v>
       </c>
       <c r="D43">
-        <v>1405</v>
+        <v>1405.0</v>
       </c>
     </row>
     <row r="44">
@@ -19069,8 +19069,8 @@
         <v>548.9</v>
       </c>
       <c r="C44">
-        <f>'FLOPs to Power'!I24</f>
-        <v>708</v>
+        <f>ROUND('FLOPs to Power'!I24,1)</f>
+        <v>708.0</v>
       </c>
       <c r="D44">
         <v>1615.8</v>
@@ -19084,8 +19084,8 @@
         <v>548.9</v>
       </c>
       <c r="C45">
-        <f>'FLOPs to Power'!I25</f>
-        <v>708</v>
+        <f>ROUND('FLOPs to Power'!I25,1)</f>
+        <v>708.0</v>
       </c>
       <c r="D45">
         <v>1858.2</v>

</xml_diff>